<commit_message>
feat: Update investor pitch deck and financial model with revised funding scenarios and projections
</commit_message>
<xml_diff>
--- a/KAILA_Founder_Grade_Package/KAILA Founder Presentation/presentation/investor-package/KAILA_Financial_Model_Starter.xlsx
+++ b/KAILA_Founder_Grade_Package/KAILA Founder Presentation/presentation/investor-package/KAILA_Financial_Model_Starter.xlsx
@@ -476,11 +476,11 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Lean pilot support target</t>
+          <t>Optional micro-budget ceiling</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>500000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="4">
@@ -726,13 +726,13 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>300000</v>
+        <v>36000</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>900000</v>
+        <v>60000</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1800000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="7">
@@ -742,13 +742,13 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>-120000</v>
+        <v>144000</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>828000</v>
+        <v>1668000</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>5490000</v>
+        <v>7170000</v>
       </c>
     </row>
   </sheetData>
@@ -790,53 +790,53 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Development</t>
+          <t>MVP polish</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>800000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Page/content boosts</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>700000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Field operations</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>300000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Legal/Admin</t>
+          <t>Admin buffer</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>200000</v>
+        <v>10000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>